<commit_message>
estimate baghdhara final rajendra
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/nagar bhaipari and estimate misc/pahiro bagh dhara/baghdhara pahiro.xlsx
+++ b/बजेट माग estimate/nagar bhaipari and estimate misc/pahiro bagh dhara/baghdhara pahiro.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4660E42B-961A-4EC0-A1EB-D7043D3B5F0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20736" windowHeight="11040" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
+    <sheet name="final estimate 300000" sheetId="13" r:id="rId2"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId2"/>
     <externalReference r:id="rId3"/>
     <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <definedNames>
     <definedName name="description_103">[1]Abstract!$B$16</definedName>
     <definedName name="description_124" localSheetId="0">#REF!</definedName>
+    <definedName name="description_124" localSheetId="1">#REF!</definedName>
     <definedName name="description_124">#REF!</definedName>
     <definedName name="description_247">[1]Abstract!$B$22</definedName>
     <definedName name="description_248">[1]Abstract!$B$23</definedName>
@@ -26,21 +27,27 @@
     <definedName name="description_276">[3]Abstract!$B$40</definedName>
     <definedName name="description_3">[1]Abstract!$B$169</definedName>
     <definedName name="description_310" localSheetId="0">#REF!</definedName>
+    <definedName name="description_310" localSheetId="1">#REF!</definedName>
     <definedName name="description_310">#REF!</definedName>
     <definedName name="description_312" localSheetId="0">#REF!</definedName>
+    <definedName name="description_312" localSheetId="1">#REF!</definedName>
     <definedName name="description_312">#REF!</definedName>
     <definedName name="description_5">[1]Abstract!$B$171</definedName>
     <definedName name="description_6" localSheetId="0">#REF!</definedName>
+    <definedName name="description_6" localSheetId="1">#REF!</definedName>
     <definedName name="description_6">#REF!</definedName>
     <definedName name="description_759">[1]Abstract!$B$278</definedName>
     <definedName name="description_781" localSheetId="0">#REF!</definedName>
+    <definedName name="description_781" localSheetId="1">#REF!</definedName>
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'final estimate 300000'!$A$1:$K$45</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'final estimate 300000'!$1:$8</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -56,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="44">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -193,10 +200,10 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
-    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -351,9 +358,9 @@
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="11" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
@@ -365,7 +372,7 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -389,14 +396,14 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -415,7 +422,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -430,7 +437,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -446,24 +453,7 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -483,15 +473,32 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Comma 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Comma 2" xfId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal 3" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="Percent 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="Normal 2" xfId="2"/>
+    <cellStyle name="Normal 3" xfId="5"/>
+    <cellStyle name="Percent 2" xfId="4"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -507,7 +514,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -601,7 +608,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Datasheet"/>
@@ -660,11 +667,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="Datasheet"/>
       <sheetName val="Abstract"/>
@@ -727,9 +731,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -767,9 +771,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -804,7 +808,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -839,7 +843,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1012,135 +1016,135 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:S49"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
-    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
-    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
-    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
-    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" style="19"/>
+    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" style="19"/>
     <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.5703125" style="19" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="9.140625" style="19"/>
+    <col min="9" max="9" width="9.5546875" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.109375" style="19"/>
     <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="19"/>
+    <col min="17" max="16384" width="9.109375" style="19"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="38"/>
-      <c r="C1" s="38"/>
-      <c r="D1" s="38"/>
-      <c r="E1" s="38"/>
-      <c r="F1" s="38"/>
-      <c r="G1" s="38"/>
-      <c r="H1" s="38"/>
-      <c r="I1" s="38"/>
-      <c r="J1" s="38"/>
-      <c r="K1" s="38"/>
-    </row>
-    <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="39" t="s">
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+    </row>
+    <row r="2" spans="1:16" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
-      <c r="K2" s="39"/>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" s="40" t="s">
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="40" t="s">
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="48" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="40"/>
-      <c r="C4" s="40"/>
-      <c r="D4" s="40"/>
-      <c r="E4" s="40"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
-      <c r="I4" s="40"/>
-      <c r="J4" s="40"/>
-      <c r="K4" s="40"/>
-    </row>
-    <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A5" s="41" t="s">
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
+    </row>
+    <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A5" s="49" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="41"/>
-      <c r="I5" s="41"/>
-      <c r="J5" s="41"/>
-      <c r="K5" s="41"/>
-    </row>
-    <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="36" t="s">
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
+    </row>
+    <row r="6" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="44" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="36"/>
-      <c r="C6" s="36"/>
-      <c r="D6" s="36"/>
-      <c r="E6" s="36"/>
-      <c r="F6" s="36"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
       <c r="G6" s="10"/>
-      <c r="H6" s="37" t="s">
+      <c r="H6" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="37"/>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
-    </row>
-    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="44" t="s">
+      <c r="I6" s="45"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="45"/>
+    </row>
+    <row r="7" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="44"/>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
       <c r="G7" s="11"/>
-      <c r="H7" s="45" t="s">
+      <c r="H7" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="I7" s="45"/>
-      <c r="J7" s="45"/>
-      <c r="K7" s="45"/>
-    </row>
-    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="I7" s="40"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="40"/>
+    </row>
+    <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="12" t="s">
         <v>6</v>
       </c>
@@ -1175,7 +1179,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:16" ht="157.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" ht="156" x14ac:dyDescent="0.3">
       <c r="A9" s="16">
         <v>1</v>
       </c>
@@ -1192,7 +1196,7 @@
       <c r="J9" s="17"/>
       <c r="K9" s="17"/>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="16"/>
       <c r="B10" s="32" t="s">
         <v>38</v>
@@ -1233,7 +1237,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="16"/>
       <c r="B11" s="32"/>
       <c r="C11" s="17">
@@ -1260,12 +1264,12 @@
       <c r="I11" s="17"/>
       <c r="J11" s="17"/>
       <c r="K11" s="17"/>
-      <c r="M11" s="49"/>
-      <c r="N11" s="49"/>
-      <c r="O11" s="49"/>
-      <c r="P11" s="49"/>
-    </row>
-    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M11" s="36"/>
+      <c r="N11" s="36"/>
+      <c r="O11" s="36"/>
+      <c r="P11" s="36"/>
+    </row>
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="34" t="s">
         <v>17</v>
@@ -1290,7 +1294,7 @@
       </c>
       <c r="K12" s="5"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="16"/>
       <c r="B13" s="32" t="s">
         <v>23</v>
@@ -1308,7 +1312,7 @@
       </c>
       <c r="K13" s="17"/>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="16"/>
       <c r="B14" s="17"/>
       <c r="C14" s="17"/>
@@ -1321,7 +1325,7 @@
       <c r="J14" s="17"/>
       <c r="K14" s="17"/>
     </row>
-    <row r="15" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
       <c r="A15" s="16">
         <v>2</v>
       </c>
@@ -1338,7 +1342,7 @@
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="16"/>
       <c r="B16" s="32" t="str">
         <f>B10</f>
@@ -1380,7 +1384,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="16"/>
       <c r="B17" s="32"/>
       <c r="C17" s="17">
@@ -1407,12 +1411,12 @@
       <c r="I17" s="17"/>
       <c r="J17" s="17"/>
       <c r="K17" s="17"/>
-      <c r="M17" s="49"/>
-      <c r="N17" s="49"/>
-      <c r="O17" s="49"/>
-      <c r="P17" s="49"/>
-    </row>
-    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M17" s="36"/>
+      <c r="N17" s="36"/>
+      <c r="O17" s="36"/>
+      <c r="P17" s="36"/>
+    </row>
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
       <c r="B18" s="34" t="s">
         <v>17</v>
@@ -1437,7 +1441,7 @@
       </c>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="16"/>
       <c r="B19" s="32" t="s">
         <v>23</v>
@@ -1455,7 +1459,7 @@
       </c>
       <c r="K19" s="17"/>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="16"/>
       <c r="B20" s="17"/>
       <c r="C20" s="17"/>
@@ -1468,7 +1472,7 @@
       <c r="J20" s="17"/>
       <c r="K20" s="17"/>
     </row>
-    <row r="21" spans="1:16" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16" ht="78" x14ac:dyDescent="0.3">
       <c r="A21" s="16">
         <v>3</v>
       </c>
@@ -1485,7 +1489,7 @@
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="16"/>
       <c r="B22" s="32" t="str">
         <f>B16</f>
@@ -1527,7 +1531,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="16"/>
       <c r="B23" s="32"/>
       <c r="C23" s="17">
@@ -1553,12 +1557,12 @@
       <c r="I23" s="17"/>
       <c r="J23" s="17"/>
       <c r="K23" s="17"/>
-      <c r="M23" s="49"/>
-      <c r="N23" s="49"/>
-      <c r="O23" s="49"/>
-      <c r="P23" s="49"/>
-    </row>
-    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M23" s="36"/>
+      <c r="N23" s="36"/>
+      <c r="O23" s="36"/>
+      <c r="P23" s="36"/>
+    </row>
+    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
       <c r="B24" s="34" t="s">
         <v>17</v>
@@ -1583,7 +1587,7 @@
       </c>
       <c r="K24" s="5"/>
     </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A25" s="16"/>
       <c r="B25" s="32" t="s">
         <v>31</v>
@@ -1601,7 +1605,7 @@
       </c>
       <c r="K25" s="17"/>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A26" s="16"/>
       <c r="B26" s="32" t="s">
         <v>32</v>
@@ -1619,7 +1623,7 @@
       </c>
       <c r="K26" s="17"/>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A27" s="16"/>
       <c r="B27" s="32" t="s">
         <v>33</v>
@@ -1637,7 +1641,7 @@
       </c>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A28" s="16"/>
       <c r="B28" s="32" t="s">
         <v>34</v>
@@ -1655,7 +1659,7 @@
       </c>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="16"/>
       <c r="B29" s="32" t="s">
         <v>35</v>
@@ -1673,7 +1677,7 @@
       </c>
       <c r="K29" s="17"/>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A30" s="16"/>
       <c r="B30" s="17"/>
       <c r="C30" s="17"/>
@@ -1686,7 +1690,7 @@
       <c r="J30" s="17"/>
       <c r="K30" s="17"/>
     </row>
-    <row r="31" spans="1:16" ht="141.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:16" ht="140.4" x14ac:dyDescent="0.3">
       <c r="A31" s="16">
         <v>4</v>
       </c>
@@ -1703,7 +1707,7 @@
       <c r="J31" s="17"/>
       <c r="K31" s="17"/>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A32" s="16"/>
       <c r="B32" s="32" t="str">
         <f>B22</f>
@@ -1745,7 +1749,7 @@
         <v>160.09797821843054</v>
       </c>
     </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A33" s="16"/>
       <c r="B33" s="32"/>
       <c r="C33" s="17">
@@ -1769,12 +1773,12 @@
       <c r="I33" s="17"/>
       <c r="J33" s="17"/>
       <c r="K33" s="17"/>
-      <c r="M33" s="49"/>
-      <c r="N33" s="49"/>
-      <c r="O33" s="49"/>
-      <c r="P33" s="49"/>
-    </row>
-    <row r="34" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M33" s="36"/>
+      <c r="N33" s="36"/>
+      <c r="O33" s="36"/>
+      <c r="P33" s="36"/>
+    </row>
+    <row r="34" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="2"/>
       <c r="B34" s="34" t="s">
         <v>17</v>
@@ -1799,7 +1803,7 @@
       </c>
       <c r="K34" s="5"/>
     </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A35" s="16"/>
       <c r="B35" s="32" t="s">
         <v>31</v>
@@ -1817,7 +1821,7 @@
       </c>
       <c r="K35" s="17"/>
     </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A36" s="16"/>
       <c r="B36" s="32" t="s">
         <v>32</v>
@@ -1835,7 +1839,7 @@
       </c>
       <c r="K36" s="17"/>
     </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A37" s="16"/>
       <c r="B37" s="32" t="s">
         <v>40</v>
@@ -1853,7 +1857,7 @@
       </c>
       <c r="K37" s="17"/>
     </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A38" s="16"/>
       <c r="B38" s="32" t="s">
         <v>41</v>
@@ -1871,7 +1875,7 @@
       </c>
       <c r="K38" s="17"/>
     </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A39" s="16"/>
       <c r="B39" s="17"/>
       <c r="C39" s="17"/>
@@ -1884,7 +1888,7 @@
       <c r="J39" s="17"/>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>5</v>
       </c>
@@ -1913,7 +1917,7 @@
       </c>
       <c r="K40" s="5"/>
     </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
       <c r="B41" s="8"/>
       <c r="C41" s="3"/>
@@ -1926,7 +1930,7 @@
       <c r="J41" s="18"/>
       <c r="K41" s="5"/>
     </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A42" s="21"/>
       <c r="B42" s="22" t="s">
         <v>22</v>
@@ -1944,7 +1948,7 @@
       </c>
       <c r="K42" s="25"/>
     </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
       <c r="M43" s="20"/>
       <c r="N43" s="20"/>
       <c r="O43" s="20"/>
@@ -1953,16 +1957,16 @@
       <c r="R43" s="20"/>
       <c r="S43" s="20"/>
     </row>
-    <row r="44" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="26"/>
       <c r="B44" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C44" s="42">
+      <c r="C44" s="37">
         <f>J42</f>
         <v>953517.4891694003</v>
       </c>
-      <c r="D44" s="43"/>
+      <c r="D44" s="38"/>
       <c r="E44" s="9">
         <v>100</v>
       </c>
@@ -1980,72 +1984,79 @@
       <c r="R44" s="19"/>
       <c r="S44" s="19"/>
     </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B45" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="C45" s="46">
+      <c r="C45" s="41">
         <v>850000</v>
       </c>
-      <c r="D45" s="47"/>
+      <c r="D45" s="42"/>
       <c r="E45" s="9"/>
     </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B46" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="C46" s="46">
+      <c r="C46" s="41">
         <f>C45-C48-C49</f>
         <v>807500</v>
       </c>
-      <c r="D46" s="47"/>
+      <c r="D46" s="42"/>
       <c r="E46" s="9">
         <f>C46/C44*100</f>
         <v>84.686438284777068</v>
       </c>
     </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B47" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="C47" s="48">
+      <c r="C47" s="43">
         <f>C44-C46</f>
         <v>146017.4891694003</v>
       </c>
-      <c r="D47" s="48"/>
+      <c r="D47" s="43"/>
       <c r="E47" s="9">
         <f>100-E46</f>
         <v>15.313561715222932</v>
       </c>
     </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="B48" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="C48" s="42">
+      <c r="C48" s="37">
         <f>C45*0.03</f>
         <v>25500</v>
       </c>
-      <c r="D48" s="43"/>
+      <c r="D48" s="38"/>
       <c r="E48" s="9">
         <v>3</v>
       </c>
     </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B49" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C49" s="42">
+      <c r="C49" s="37">
         <f>C45*0.02</f>
         <v>17000</v>
       </c>
-      <c r="D49" s="43"/>
+      <c r="D49" s="38"/>
       <c r="E49" s="9">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="C48:D48"/>
     <mergeCell ref="C49:D49"/>
     <mergeCell ref="A7:F7"/>
@@ -2054,13 +2065,6 @@
     <mergeCell ref="C45:D45"/>
     <mergeCell ref="C46:D46"/>
     <mergeCell ref="C47:D47"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A5:K5"/>
   </mergeCells>
   <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
@@ -2071,4 +2075,941 @@
     <brk id="30" max="10" man="1"/>
   </rowBreaks>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:S45"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="4.6640625" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.88671875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5546875" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.33203125" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" style="19"/>
+    <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5546875" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.6640625" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.109375" style="19"/>
+    <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.109375" style="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" s="46" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+    </row>
+    <row r="2" spans="1:16" ht="22.8" x14ac:dyDescent="0.3">
+      <c r="A2" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3" s="48" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="48" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
+    </row>
+    <row r="5" spans="1:16" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A5" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
+    </row>
+    <row r="6" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="45"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="45"/>
+    </row>
+    <row r="7" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="39" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="40" t="s">
+        <v>43</v>
+      </c>
+      <c r="I7" s="40"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="40"/>
+    </row>
+    <row r="8" spans="1:16" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="156" x14ac:dyDescent="0.3">
+      <c r="A9" s="16">
+        <v>1</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A10" s="16"/>
+      <c r="B10" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="D10" s="33">
+        <f>D29</f>
+        <v>15</v>
+      </c>
+      <c r="E10" s="33">
+        <f>F29/2</f>
+        <v>1.6</v>
+      </c>
+      <c r="F10" s="33">
+        <v>1.5</v>
+      </c>
+      <c r="G10" s="33">
+        <f>PRODUCT(C10:F10)</f>
+        <v>18</v>
+      </c>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="M10" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N10" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O10" s="33"/>
+      <c r="P10" s="33">
+        <f>PI()*M10*SQRT(M10^2+N10^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
+      <c r="B11" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="6">
+        <f>SUM(G10:G10)</f>
+        <v>18</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I11" s="6">
+        <v>62.95</v>
+      </c>
+      <c r="J11" s="18">
+        <f>G11*I11</f>
+        <v>1133.1000000000001</v>
+      </c>
+      <c r="K11" s="5"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A12" s="16"/>
+      <c r="B12" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="18">
+        <f>0.13*G11*(18612)/360</f>
+        <v>120.97799999999998</v>
+      </c>
+      <c r="K12" s="17"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A13" s="16"/>
+      <c r="B13" s="17"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+    </row>
+    <row r="14" spans="1:16" ht="109.2" x14ac:dyDescent="0.3">
+      <c r="A14" s="16">
+        <v>2</v>
+      </c>
+      <c r="B14" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A15" s="16"/>
+      <c r="B15" s="32" t="str">
+        <f>B10</f>
+        <v>-for plum wall</v>
+      </c>
+      <c r="C15" s="17">
+        <v>1</v>
+      </c>
+      <c r="D15" s="33">
+        <f>D20</f>
+        <v>15</v>
+      </c>
+      <c r="E15" s="33">
+        <f>E20</f>
+        <v>1.6</v>
+      </c>
+      <c r="F15" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G15" s="33">
+        <f>PRODUCT(C15:F15)</f>
+        <v>3.5999999999999996</v>
+      </c>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="17"/>
+      <c r="K15" s="17"/>
+      <c r="M15" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N15" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O15" s="33"/>
+      <c r="P15" s="33">
+        <f>PI()*M15*SQRT(M15^2+N15^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="2"/>
+      <c r="B16" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="6">
+        <f>SUM(G15:G15)</f>
+        <v>3.5999999999999996</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I16" s="6">
+        <v>4458.5200000000004</v>
+      </c>
+      <c r="J16" s="18">
+        <f>G16*I16</f>
+        <v>16050.672</v>
+      </c>
+      <c r="K16" s="5"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A17" s="16"/>
+      <c r="B17" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="18">
+        <f>0.13*G16*(14817.6)/5</f>
+        <v>1386.9273599999999</v>
+      </c>
+      <c r="K17" s="17"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A18" s="16"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+    </row>
+    <row r="19" spans="1:16" ht="78" x14ac:dyDescent="0.3">
+      <c r="A19" s="16">
+        <v>3</v>
+      </c>
+      <c r="B19" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A20" s="16"/>
+      <c r="B20" s="32" t="str">
+        <f>B15</f>
+        <v>-for plum wall</v>
+      </c>
+      <c r="C20" s="17">
+        <v>1</v>
+      </c>
+      <c r="D20" s="33">
+        <f>D29</f>
+        <v>15</v>
+      </c>
+      <c r="E20" s="33">
+        <f>F29/2</f>
+        <v>1.6</v>
+      </c>
+      <c r="F20" s="33">
+        <v>0.05</v>
+      </c>
+      <c r="G20" s="33">
+        <f>PRODUCT(C20:F20)</f>
+        <v>1.2000000000000002</v>
+      </c>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="M20" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N20" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O20" s="33"/>
+      <c r="P20" s="33">
+        <f>PI()*M20*SQRT(M20^2+N20^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="2"/>
+      <c r="B21" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C21" s="3"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="5"/>
+      <c r="G21" s="6">
+        <f>SUM(G20:G20)</f>
+        <v>1.2000000000000002</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I21" s="6">
+        <v>10964.46</v>
+      </c>
+      <c r="J21" s="18">
+        <f>G21*I21</f>
+        <v>13157.352000000001</v>
+      </c>
+      <c r="K21" s="5"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A22" s="16"/>
+      <c r="B22" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="18">
+        <f>0.13*G21*(53818.03)/15</f>
+        <v>559.70751200000018</v>
+      </c>
+      <c r="K22" s="17"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A23" s="16"/>
+      <c r="B23" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="18">
+        <f>0.13*G21*(21432.6)/15</f>
+        <v>222.89904000000004</v>
+      </c>
+      <c r="K23" s="17"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A24" s="16"/>
+      <c r="B24" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="18">
+        <f>0.13*G21*(25719.12+13573.98+4286.52)/15</f>
+        <v>453.228048</v>
+      </c>
+      <c r="K24" s="17"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A25" s="16"/>
+      <c r="B25" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="18">
+        <f>0.13*G21*(6325.7)/15</f>
+        <v>65.78728000000001</v>
+      </c>
+      <c r="K25" s="17"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A26" s="16"/>
+      <c r="B26" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="18">
+        <f>0.13*G21*(310)/5</f>
+        <v>9.6720000000000006</v>
+      </c>
+      <c r="K26" s="17"/>
+    </row>
+    <row r="27" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A27" s="16"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+    </row>
+    <row r="28" spans="1:16" ht="140.4" x14ac:dyDescent="0.3">
+      <c r="A28" s="16">
+        <v>4</v>
+      </c>
+      <c r="B28" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+    </row>
+    <row r="29" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A29" s="16"/>
+      <c r="B29" s="32" t="str">
+        <f>B20</f>
+        <v>-for plum wall</v>
+      </c>
+      <c r="C29" s="17">
+        <v>1</v>
+      </c>
+      <c r="D29" s="33">
+        <v>15</v>
+      </c>
+      <c r="E29" s="33">
+        <f>((F29/2)+0.5)/2</f>
+        <v>1.05</v>
+      </c>
+      <c r="F29" s="33">
+        <v>3.2</v>
+      </c>
+      <c r="G29" s="33">
+        <f>PRODUCT(C29:F29)</f>
+        <v>50.400000000000006</v>
+      </c>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17"/>
+      <c r="M29" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N29" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O29" s="33"/>
+      <c r="P29" s="33">
+        <f>PI()*M29*SQRT(M29^2+N29^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="2"/>
+      <c r="B30" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="3"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="5"/>
+      <c r="F30" s="5"/>
+      <c r="G30" s="6">
+        <f>SUM(G29:G29)</f>
+        <v>50.400000000000006</v>
+      </c>
+      <c r="H30" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I30" s="6">
+        <v>9860.43</v>
+      </c>
+      <c r="J30" s="18">
+        <f>G30*I30</f>
+        <v>496965.67200000008</v>
+      </c>
+      <c r="K30" s="5"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A31" s="16"/>
+      <c r="B31" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="18">
+        <f>0.13*G30*(22152.7)/10</f>
+        <v>14514.449040000003</v>
+      </c>
+      <c r="K31" s="17"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A32" s="16"/>
+      <c r="B32" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="18">
+        <f>0.13*G30*(9525.6)/10</f>
+        <v>6241.1731200000013</v>
+      </c>
+      <c r="K32" s="17"/>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A33" s="16"/>
+      <c r="B33" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="18">
+        <f>0.13*G30*(11331.936)/10</f>
+        <v>7424.6844672000007</v>
+      </c>
+      <c r="K33" s="17"/>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A34" s="16"/>
+      <c r="B34" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="18">
+        <f>0.13*G30*(10954.44+5228.496+2286.144)/10</f>
+        <v>12100.941216000003</v>
+      </c>
+      <c r="K34" s="17"/>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A35" s="16"/>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
+      <c r="D35" s="17"/>
+      <c r="E35" s="17"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="17"/>
+      <c r="H35" s="17"/>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17"/>
+      <c r="K35" s="17"/>
+    </row>
+    <row r="36" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="2">
+        <v>5</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="3">
+        <v>1</v>
+      </c>
+      <c r="D36" s="4"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="7">
+        <f t="shared" ref="G36" si="0">PRODUCT(C36:F36)</f>
+        <v>1</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I36" s="6">
+        <v>500</v>
+      </c>
+      <c r="J36" s="7">
+        <f>G36*I36</f>
+        <v>500</v>
+      </c>
+      <c r="K36" s="5"/>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A37" s="2"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="5"/>
+      <c r="F37" s="5"/>
+      <c r="G37" s="6"/>
+      <c r="H37" s="7"/>
+      <c r="I37" s="6"/>
+      <c r="J37" s="18"/>
+      <c r="K37" s="5"/>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A38" s="21"/>
+      <c r="B38" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C38" s="23"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="18"/>
+      <c r="J38" s="18">
+        <f>SUM(J9:J36)</f>
+        <v>570907.24308320007</v>
+      </c>
+      <c r="K38" s="25"/>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="M39" s="20"/>
+      <c r="N39" s="20"/>
+      <c r="O39" s="20"/>
+      <c r="P39" s="20"/>
+      <c r="Q39" s="20"/>
+      <c r="R39" s="20"/>
+      <c r="S39" s="20"/>
+    </row>
+    <row r="40" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="26"/>
+      <c r="B40" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40" s="37">
+        <f>J38</f>
+        <v>570907.24308320007</v>
+      </c>
+      <c r="D40" s="38"/>
+      <c r="E40" s="9">
+        <v>100</v>
+      </c>
+      <c r="F40" s="26"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="26"/>
+      <c r="I40" s="29"/>
+      <c r="J40" s="30"/>
+      <c r="K40" s="31"/>
+      <c r="M40" s="19"/>
+      <c r="N40" s="19"/>
+      <c r="O40" s="19"/>
+      <c r="P40" s="19"/>
+      <c r="Q40" s="19"/>
+      <c r="R40" s="19"/>
+      <c r="S40" s="19"/>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="B41" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="C41" s="41">
+        <v>300000</v>
+      </c>
+      <c r="D41" s="42"/>
+      <c r="E41" s="9"/>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="B42" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C42" s="41">
+        <f>C41-C44-C45</f>
+        <v>285000</v>
+      </c>
+      <c r="D42" s="42"/>
+      <c r="E42" s="9">
+        <f>C42/C40*100</f>
+        <v>49.92054374031931</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="B43" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C43" s="43">
+        <f>C40-C42</f>
+        <v>285907.24308320007</v>
+      </c>
+      <c r="D43" s="43"/>
+      <c r="E43" s="9">
+        <f>100-E42</f>
+        <v>50.07945625968069</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="B44" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="C44" s="37">
+        <f>C41*0.03</f>
+        <v>9000</v>
+      </c>
+      <c r="D44" s="38"/>
+      <c r="E44" s="9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="B45" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C45" s="37">
+        <f>C41*0.02</f>
+        <v>6000</v>
+      </c>
+      <c r="D45" s="38"/>
+      <c r="E45" s="9">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C45:D45"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+  </mergeCells>
+  <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
+  </headerFooter>
+  <rowBreaks count="1" manualBreakCount="1">
+    <brk id="27" max="10" man="1"/>
+  </rowBreaks>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
tallo nangle dware chihan paati
</commit_message>
<xml_diff>
--- a/बजेट माग estimate/nagar bhaipari and estimate misc/pahiro bagh dhara/baghdhara pahiro.xlsx
+++ b/बजेट माग estimate/nagar bhaipari and estimate misc/pahiro bagh dhara/baghdhara pahiro.xlsx
@@ -3,22 +3,24 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70E5AB57-C666-4FC4-8343-E30F5FCEEF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF065EBE-E60A-4A4C-A613-ED3DE1B3E3EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="estimate" sheetId="12" r:id="rId1"/>
     <sheet name="final estimate 300000" sheetId="13" r:id="rId2"/>
+    <sheet name="final estimate 150000" sheetId="14" r:id="rId3"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
     <externalReference r:id="rId4"/>
     <externalReference r:id="rId5"/>
+    <externalReference r:id="rId6"/>
   </externalReferences>
   <definedNames>
     <definedName name="description_103">[1]Abstract!$B$16</definedName>
     <definedName name="description_124" localSheetId="0">#REF!</definedName>
+    <definedName name="description_124" localSheetId="2">#REF!</definedName>
     <definedName name="description_124" localSheetId="1">#REF!</definedName>
     <definedName name="description_124">#REF!</definedName>
     <definedName name="description_247">[1]Abstract!$B$22</definedName>
@@ -28,24 +30,30 @@
     <definedName name="description_276">[3]Abstract!$B$40</definedName>
     <definedName name="description_3">[1]Abstract!$B$169</definedName>
     <definedName name="description_310" localSheetId="0">#REF!</definedName>
+    <definedName name="description_310" localSheetId="2">#REF!</definedName>
     <definedName name="description_310" localSheetId="1">#REF!</definedName>
     <definedName name="description_310">#REF!</definedName>
     <definedName name="description_312" localSheetId="0">#REF!</definedName>
+    <definedName name="description_312" localSheetId="2">#REF!</definedName>
     <definedName name="description_312" localSheetId="1">#REF!</definedName>
     <definedName name="description_312">#REF!</definedName>
     <definedName name="description_5">[1]Abstract!$B$171</definedName>
     <definedName name="description_6" localSheetId="0">#REF!</definedName>
+    <definedName name="description_6" localSheetId="2">#REF!</definedName>
     <definedName name="description_6" localSheetId="1">#REF!</definedName>
     <definedName name="description_6">#REF!</definedName>
     <definedName name="description_759">[1]Abstract!$B$278</definedName>
     <definedName name="description_781" localSheetId="0">#REF!</definedName>
+    <definedName name="description_781" localSheetId="2">#REF!</definedName>
     <definedName name="description_781" localSheetId="1">#REF!</definedName>
     <definedName name="description_781">#REF!</definedName>
     <definedName name="description_783">[1]Abstract!$B$301</definedName>
     <definedName name="description_784">[3]Abstract!$B$300</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">estimate!$A$1:$K$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'final estimate 150000'!$A$1:$K$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'final estimate 300000'!$A$1:$K$44</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">estimate!$1:$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'final estimate 150000'!$1:$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'final estimate 300000'!$1:$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -66,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="45">
   <si>
     <t>Government of Nepal</t>
   </si>
@@ -2997,4 +3005,921 @@
     <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14ABBD4D-DE9C-426B-97CC-F08821681F39}">
+  <dimension ref="A1:S44"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.7109375" style="19" customWidth="1"/>
+    <col min="2" max="2" width="30.85546875" style="19" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" style="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.42578125" style="19" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" style="19" customWidth="1"/>
+    <col min="6" max="6" width="7.28515625" style="19" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="19"/>
+    <col min="8" max="8" width="5" style="19" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.5703125" style="19" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7109375" style="19" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" style="19"/>
+    <col min="13" max="16" width="0" style="19" hidden="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="19"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="46" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+    </row>
+    <row r="2" spans="1:16" ht="22.5" x14ac:dyDescent="0.25">
+      <c r="A2" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="48" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
+      <c r="E3" s="48"/>
+      <c r="F3" s="48"/>
+      <c r="G3" s="48"/>
+      <c r="H3" s="48"/>
+      <c r="I3" s="48"/>
+      <c r="J3" s="48"/>
+      <c r="K3" s="48"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="48" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
+    </row>
+    <row r="5" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A5" s="49" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
+      <c r="F5" s="49"/>
+      <c r="G5" s="49"/>
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
+    </row>
+    <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="44" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="44"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="45" t="s">
+        <v>28</v>
+      </c>
+      <c r="I6" s="45"/>
+      <c r="J6" s="45"/>
+      <c r="K6" s="45"/>
+    </row>
+    <row r="7" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="39" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="39"/>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="39"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="40" t="s">
+        <v>44</v>
+      </c>
+      <c r="I7" s="40"/>
+      <c r="J7" s="40"/>
+      <c r="K7" s="40"/>
+    </row>
+    <row r="8" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="174.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="16">
+        <v>1</v>
+      </c>
+      <c r="B9" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A10" s="16"/>
+      <c r="B10" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="17">
+        <v>0.5</v>
+      </c>
+      <c r="D10" s="33">
+        <f>D28</f>
+        <v>8.381590978360256</v>
+      </c>
+      <c r="E10" s="33">
+        <f>F28/2</f>
+        <v>1.5</v>
+      </c>
+      <c r="F10" s="33">
+        <v>1.5</v>
+      </c>
+      <c r="G10" s="33">
+        <f>PRODUCT(C10:F10)</f>
+        <v>9.4292898506552874</v>
+      </c>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="M10" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N10" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O10" s="33"/>
+      <c r="P10" s="33">
+        <f>PI()*M10*SQRT(M10^2+N10^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="6">
+        <f>SUM(G10:G10)</f>
+        <v>9.4292898506552874</v>
+      </c>
+      <c r="H11" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I11" s="6">
+        <v>748.9</v>
+      </c>
+      <c r="J11" s="18">
+        <f>G11*I11</f>
+        <v>7061.5951691557448</v>
+      </c>
+      <c r="K11" s="5"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" s="16"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
+      <c r="K12" s="17"/>
+    </row>
+    <row r="13" spans="1:16" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A13" s="16">
+        <v>2</v>
+      </c>
+      <c r="B13" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
+      <c r="K13" s="17"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A14" s="16"/>
+      <c r="B14" s="32" t="str">
+        <f>B10</f>
+        <v>-for plum wall</v>
+      </c>
+      <c r="C14" s="17">
+        <v>1</v>
+      </c>
+      <c r="D14" s="33">
+        <f>D19</f>
+        <v>8.381590978360256</v>
+      </c>
+      <c r="E14" s="33">
+        <f>E19</f>
+        <v>1.5</v>
+      </c>
+      <c r="F14" s="33">
+        <v>0.15</v>
+      </c>
+      <c r="G14" s="33">
+        <f>PRODUCT(C14:F14)</f>
+        <v>1.8858579701310574</v>
+      </c>
+      <c r="H14" s="17"/>
+      <c r="I14" s="17"/>
+      <c r="J14" s="17"/>
+      <c r="K14" s="17"/>
+      <c r="M14" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N14" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O14" s="33"/>
+      <c r="P14" s="33">
+        <f>PI()*M14*SQRT(M14^2+N14^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2"/>
+      <c r="B15" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="5"/>
+      <c r="G15" s="6">
+        <f>SUM(G14:G14)</f>
+        <v>1.8858579701310574</v>
+      </c>
+      <c r="H15" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I15" s="6">
+        <v>4458.5200000000004</v>
+      </c>
+      <c r="J15" s="18">
+        <f>G15*I15</f>
+        <v>8408.1354769887221</v>
+      </c>
+      <c r="K15" s="5"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16" s="16"/>
+      <c r="B16" s="32" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="18">
+        <f>0.13*G15*(14817.6)/5</f>
+        <v>726.54111551356289</v>
+      </c>
+      <c r="K16" s="17"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" s="16"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+    </row>
+    <row r="18" spans="1:16" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="16">
+        <v>3</v>
+      </c>
+      <c r="B18" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A19" s="16"/>
+      <c r="B19" s="32" t="str">
+        <f>B14</f>
+        <v>-for plum wall</v>
+      </c>
+      <c r="C19" s="17">
+        <v>1</v>
+      </c>
+      <c r="D19" s="33">
+        <f>D28</f>
+        <v>8.381590978360256</v>
+      </c>
+      <c r="E19" s="33">
+        <f>F28/2</f>
+        <v>1.5</v>
+      </c>
+      <c r="F19" s="33">
+        <v>0.05</v>
+      </c>
+      <c r="G19" s="33">
+        <f>PRODUCT(C19:F19)</f>
+        <v>0.6286193233770192</v>
+      </c>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
+      <c r="M19" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N19" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O19" s="33"/>
+      <c r="P19" s="33">
+        <f>PI()*M19*SQRT(M19^2+N19^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2"/>
+      <c r="B20" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="6">
+        <f>SUM(G19:G19)</f>
+        <v>0.6286193233770192</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I20" s="6">
+        <v>10964.46</v>
+      </c>
+      <c r="J20" s="18">
+        <f>G20*I20</f>
+        <v>6892.4714263943915</v>
+      </c>
+      <c r="K20" s="5"/>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A21" s="16"/>
+      <c r="B21" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
+      <c r="J21" s="18">
+        <f>0.13*G20*(53818.03)/15</f>
+        <v>293.20246456872906</v>
+      </c>
+      <c r="K21" s="17"/>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A22" s="16"/>
+      <c r="B22" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="17"/>
+      <c r="I22" s="17"/>
+      <c r="J22" s="18">
+        <f>0.13*G20*(21432.6)/15</f>
+        <v>116.7655364218226</v>
+      </c>
+      <c r="K22" s="17"/>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A23" s="16"/>
+      <c r="B23" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="18">
+        <f>0.13*G20*(25719.12+13573.98+4286.52)/15</f>
+        <v>237.4232573910393</v>
+      </c>
+      <c r="K23" s="17"/>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A24" s="16"/>
+      <c r="B24" s="32" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="18">
+        <f>0.13*G20*(6325.7)/15</f>
+        <v>34.462629533678758</v>
+      </c>
+      <c r="K24" s="17"/>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A25" s="16"/>
+      <c r="B25" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="18">
+        <f>0.13*G20*(310)/5</f>
+        <v>5.0666717464187752</v>
+      </c>
+      <c r="K25" s="17"/>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A26" s="16"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="17"/>
+      <c r="I26" s="17"/>
+      <c r="J26" s="17"/>
+      <c r="K26" s="17"/>
+    </row>
+    <row r="27" spans="1:16" ht="141.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="16">
+        <v>4</v>
+      </c>
+      <c r="B27" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="17"/>
+      <c r="H27" s="17"/>
+      <c r="I27" s="17"/>
+      <c r="J27" s="17"/>
+      <c r="K27" s="17"/>
+    </row>
+    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A28" s="16"/>
+      <c r="B28" s="32" t="str">
+        <f>B19</f>
+        <v>-for plum wall</v>
+      </c>
+      <c r="C28" s="17">
+        <v>1</v>
+      </c>
+      <c r="D28" s="33">
+        <f>27.5/3.281</f>
+        <v>8.381590978360256</v>
+      </c>
+      <c r="E28" s="33">
+        <f>((F28/2)+0.45)/2</f>
+        <v>0.97499999999999998</v>
+      </c>
+      <c r="F28" s="33">
+        <v>3</v>
+      </c>
+      <c r="G28" s="33">
+        <f>PRODUCT(C28:F28)</f>
+        <v>24.51615361170375</v>
+      </c>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="M28" s="33">
+        <f>7</f>
+        <v>7</v>
+      </c>
+      <c r="N28" s="33">
+        <f>2</f>
+        <v>2</v>
+      </c>
+      <c r="O28" s="33"/>
+      <c r="P28" s="33">
+        <f>PI()*M28*SQRT(M28^2+N28^2)</f>
+        <v>160.09797821843054</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2"/>
+      <c r="B29" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="3"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="6">
+        <f>SUM(G28:G28)</f>
+        <v>24.51615361170375</v>
+      </c>
+      <c r="H29" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I29" s="6">
+        <v>9860.43</v>
+      </c>
+      <c r="J29" s="18">
+        <f>G29*I29</f>
+        <v>241739.81655745202</v>
+      </c>
+      <c r="K29" s="5"/>
+    </row>
+    <row r="30" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A30" s="16"/>
+      <c r="B30" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="18">
+        <f>0.13*G29*(22152.7)/10</f>
+        <v>7060.286949481866</v>
+      </c>
+      <c r="K30" s="17"/>
+    </row>
+    <row r="31" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A31" s="16"/>
+      <c r="B31" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="17"/>
+      <c r="I31" s="17"/>
+      <c r="J31" s="18">
+        <f>0.13*G29*(9525.6)/10</f>
+        <v>3035.903946967388</v>
+      </c>
+      <c r="K31" s="17"/>
+    </row>
+    <row r="32" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A32" s="16"/>
+      <c r="B32" s="32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="17"/>
+      <c r="I32" s="17"/>
+      <c r="J32" s="18">
+        <f>0.13*G29*(11331.936)/10</f>
+        <v>3611.6012880219446</v>
+      </c>
+      <c r="K32" s="17"/>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A33" s="16"/>
+      <c r="B33" s="32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="17"/>
+      <c r="I33" s="17"/>
+      <c r="J33" s="18">
+        <f>0.13*G29*(10954.44+5228.496+2286.144)/10</f>
+        <v>5886.2804305089921</v>
+      </c>
+      <c r="K33" s="17"/>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A34" s="16"/>
+      <c r="B34" s="17"/>
+      <c r="C34" s="17"/>
+      <c r="D34" s="17"/>
+      <c r="E34" s="17"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="17"/>
+      <c r="H34" s="17"/>
+      <c r="I34" s="17"/>
+      <c r="J34" s="17"/>
+      <c r="K34" s="17"/>
+    </row>
+    <row r="35" spans="1:19" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>5</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" s="3">
+        <v>1</v>
+      </c>
+      <c r="D35" s="4"/>
+      <c r="E35" s="5"/>
+      <c r="F35" s="5"/>
+      <c r="G35" s="7">
+        <f t="shared" ref="G35" si="0">PRODUCT(C35:F35)</f>
+        <v>1</v>
+      </c>
+      <c r="H35" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I35" s="6">
+        <v>500</v>
+      </c>
+      <c r="J35" s="7">
+        <f>G35*I35</f>
+        <v>500</v>
+      </c>
+      <c r="K35" s="5"/>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A36" s="2"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="5"/>
+      <c r="F36" s="5"/>
+      <c r="G36" s="6"/>
+      <c r="H36" s="7"/>
+      <c r="I36" s="6"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="5"/>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A37" s="21"/>
+      <c r="B37" s="22" t="s">
+        <v>22</v>
+      </c>
+      <c r="C37" s="23"/>
+      <c r="D37" s="24"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="18"/>
+      <c r="J37" s="18">
+        <f>SUM(J9:J35)</f>
+        <v>285609.55292014638</v>
+      </c>
+      <c r="K37" s="25"/>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="M38" s="20"/>
+      <c r="N38" s="20"/>
+      <c r="O38" s="20"/>
+      <c r="P38" s="20"/>
+      <c r="Q38" s="20"/>
+      <c r="R38" s="20"/>
+      <c r="S38" s="20"/>
+    </row>
+    <row r="39" spans="1:19" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="26"/>
+      <c r="B39" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C39" s="37">
+        <f>J37</f>
+        <v>285609.55292014638</v>
+      </c>
+      <c r="D39" s="38"/>
+      <c r="E39" s="9">
+        <v>100</v>
+      </c>
+      <c r="F39" s="26"/>
+      <c r="G39" s="28"/>
+      <c r="H39" s="26"/>
+      <c r="I39" s="29"/>
+      <c r="J39" s="30"/>
+      <c r="K39" s="31"/>
+      <c r="M39" s="19"/>
+      <c r="N39" s="19"/>
+      <c r="O39" s="19"/>
+      <c r="P39" s="19"/>
+      <c r="Q39" s="19"/>
+      <c r="R39" s="19"/>
+      <c r="S39" s="19"/>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B40" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="C40" s="41">
+        <v>150000</v>
+      </c>
+      <c r="D40" s="42"/>
+      <c r="E40" s="9"/>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B41" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" s="41">
+        <f>C40-C43-C44</f>
+        <v>142500</v>
+      </c>
+      <c r="D41" s="42"/>
+      <c r="E41" s="9">
+        <f>C41/C39*100</f>
+        <v>49.893289122525111</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B42" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C42" s="43">
+        <f>C39-C41</f>
+        <v>143109.55292014638</v>
+      </c>
+      <c r="D42" s="43"/>
+      <c r="E42" s="9">
+        <f>100-E41</f>
+        <v>50.106710877474889</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B43" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="C43" s="37">
+        <f>C40*0.03</f>
+        <v>4500</v>
+      </c>
+      <c r="D43" s="38"/>
+      <c r="E43" s="9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="B44" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="C44" s="37">
+        <f>C40*0.02</f>
+        <v>3000</v>
+      </c>
+      <c r="D44" s="38"/>
+      <c r="E44" s="9">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A4:K4"/>
+    <mergeCell ref="A5:K5"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="C41:D41"/>
+    <mergeCell ref="C42:D42"/>
+  </mergeCells>
+  <pageMargins left="0.70866141732283505" right="0.70866141732283505" top="0.74803149606299202" bottom="0.74803149606299202" header="0.31496062992126" footer="0.31496062992126"/>
+  <pageSetup paperSize="9" scale="80" orientation="portrait" verticalDpi="1200" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;LPrepared By:&amp;CChecked By:&amp;RApproved By:</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>